<commit_message>
check species match by alternate name, and change some garwood names to the most recent forestgeo name
</commit_message>
<xml_diff>
--- a/splists_out/Lianas_Species_complete_list_WCVP_CHANGES_2026-03-03.xlsx
+++ b/splists_out/Lianas_Species_complete_list_WCVP_CHANGES_2026-03-03.xlsx
@@ -351,7 +351,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:AD22"/>
+  <dimension ref="A1:AN22"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" s="1" customFormat="1">
@@ -367,140 +367,190 @@
       </c>
       <c r="C1" s="1" t="inlineStr">
         <is>
+          <t>binomialFormer</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>binomialplus</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>binomialplusFormer</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
           <t>orig_family</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
+      <c r="G1" s="1" t="inlineStr">
         <is>
           <t>orig_genus</t>
         </is>
       </c>
-      <c r="E1" s="1" t="inlineStr">
+      <c r="H1" s="1" t="inlineStr">
         <is>
           <t>orig_species</t>
         </is>
       </c>
-      <c r="F1" s="1" t="inlineStr">
+      <c r="I1" s="1" t="inlineStr">
+        <is>
+          <t>Subspecies</t>
+        </is>
+      </c>
+      <c r="J1" s="1" t="inlineStr">
         <is>
           <t>orig_author</t>
         </is>
       </c>
-      <c r="G1" s="1" t="inlineStr">
+      <c r="K1" s="1" t="inlineStr">
+        <is>
+          <t>FamilyFormer</t>
+        </is>
+      </c>
+      <c r="L1" s="1" t="inlineStr">
+        <is>
+          <t>GenusFormer</t>
+        </is>
+      </c>
+      <c r="M1" s="1" t="inlineStr">
+        <is>
+          <t>SpeciesOnlyFormer</t>
+        </is>
+      </c>
+      <c r="N1" s="1" t="inlineStr">
+        <is>
+          <t>SubspeciesFormer</t>
+        </is>
+      </c>
+      <c r="O1" s="1" t="inlineStr">
+        <is>
+          <t>AuthorityFormer</t>
+        </is>
+      </c>
+      <c r="P1" s="1" t="inlineStr">
+        <is>
+          <t>isbci</t>
+        </is>
+      </c>
+      <c r="Q1" s="1" t="inlineStr">
         <is>
           <t>orig_infraspecies_rank</t>
         </is>
       </c>
-      <c r="H1" s="1" t="inlineStr">
+      <c r="R1" s="1" t="inlineStr">
         <is>
           <t>orig_infraspecies</t>
         </is>
       </c>
-      <c r="I1" s="1" t="inlineStr">
+      <c r="S1" s="1" t="inlineStr">
         <is>
           <t>orig_binomial</t>
         </is>
       </c>
-      <c r="J1" s="1" t="inlineStr">
+      <c r="T1" s="1" t="inlineStr">
         <is>
           <t>wcvp_matched_name</t>
         </is>
       </c>
-      <c r="K1" s="1" t="inlineStr">
+      <c r="U1" s="1" t="inlineStr">
         <is>
           <t>wcvp_matched_authors</t>
         </is>
       </c>
-      <c r="L1" s="1" t="inlineStr">
+      <c r="V1" s="1" t="inlineStr">
         <is>
           <t>wcvp_matched_rank</t>
         </is>
       </c>
-      <c r="M1" s="1" t="inlineStr">
+      <c r="W1" s="1" t="inlineStr">
         <is>
           <t>wcvp_matched_status</t>
         </is>
       </c>
-      <c r="N1" s="1" t="inlineStr">
+      <c r="X1" s="1" t="inlineStr">
         <is>
           <t>wcvp_matched_plant_name_id</t>
         </is>
       </c>
-      <c r="O1" s="1" t="inlineStr">
+      <c r="Y1" s="1" t="inlineStr">
         <is>
           <t>wcvp_matched_ipni_id</t>
         </is>
       </c>
-      <c r="P1" s="1" t="inlineStr">
+      <c r="Z1" s="1" t="inlineStr">
         <is>
           <t>match_similarity</t>
         </is>
       </c>
-      <c r="Q1" s="1" t="inlineStr">
+      <c r="AA1" s="1" t="inlineStr">
         <is>
           <t>wcvp_accepted_plant_name_id</t>
         </is>
       </c>
-      <c r="R1" s="1" t="inlineStr">
+      <c r="AB1" s="1" t="inlineStr">
         <is>
           <t>wcvp_accepted_powo_id</t>
         </is>
       </c>
-      <c r="S1" s="1" t="inlineStr">
+      <c r="AC1" s="1" t="inlineStr">
         <is>
           <t>wcvp_accepted_ipni_id</t>
         </is>
       </c>
-      <c r="T1" s="1" t="inlineStr">
+      <c r="AD1" s="1" t="inlineStr">
         <is>
           <t>wcvp_accepted_name</t>
         </is>
       </c>
-      <c r="U1" s="1" t="inlineStr">
+      <c r="AE1" s="1" t="inlineStr">
         <is>
           <t>wcvp_accepted_name_genus</t>
         </is>
       </c>
-      <c r="V1" s="1" t="inlineStr">
+      <c r="AF1" s="1" t="inlineStr">
         <is>
           <t>wcvp_accepted_name_species</t>
         </is>
       </c>
-      <c r="W1" s="1" t="inlineStr">
+      <c r="AG1" s="1" t="inlineStr">
         <is>
           <t>wcvp_accepted_name_rank</t>
         </is>
       </c>
-      <c r="X1" s="1" t="inlineStr">
+      <c r="AH1" s="1" t="inlineStr">
         <is>
           <t>wcvp_accepted_family</t>
         </is>
       </c>
-      <c r="Y1" s="1" t="inlineStr">
+      <c r="AI1" s="1" t="inlineStr">
         <is>
           <t>wcvp_accepted_name_infraspecific_rank</t>
         </is>
       </c>
-      <c r="Z1" s="1" t="inlineStr">
+      <c r="AJ1" s="1" t="inlineStr">
         <is>
           <t>wcvp_accepted_name_infraspecies</t>
         </is>
       </c>
-      <c r="AA1" s="1" t="inlineStr">
+      <c r="AK1" s="1" t="inlineStr">
         <is>
           <t>wcvp_accepted_author</t>
         </is>
       </c>
-      <c r="AB1" s="1" t="inlineStr">
+      <c r="AL1" s="1" t="inlineStr">
         <is>
           <t>wcvp_accepted_authority</t>
         </is>
       </c>
-      <c r="AC1" s="1" t="inlineStr">
+      <c r="AM1" s="1" t="inlineStr">
         <is>
           <t>wcvp_lifeform_description</t>
         </is>
       </c>
-      <c r="AD1" s="1" t="inlineStr">
+      <c r="AN1" s="1" t="inlineStr">
         <is>
           <t>origmatches</t>
         </is>
@@ -519,114 +569,132 @@
       </c>
       <c r="C2" t="inlineStr">
         <is>
+          <t>NA NA</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>Anthodon panamense</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>NA NA</t>
+        </is>
+      </c>
+      <c r="F2" t="inlineStr">
+        <is>
           <t>Celastraceae</t>
         </is>
       </c>
-      <c r="D2" t="inlineStr">
+      <c r="G2" t="inlineStr">
         <is>
           <t>Anthodon</t>
         </is>
       </c>
-      <c r="E2" t="inlineStr">
+      <c r="H2" t="inlineStr">
         <is>
           <t>panamense</t>
         </is>
       </c>
-      <c r="F2" t="inlineStr">
+      <c r="J2" t="inlineStr">
         <is>
           <t>A.C. Sm.</t>
         </is>
       </c>
-      <c r="I2" t="inlineStr">
+      <c r="P2" t="b">
+        <v>1</v>
+      </c>
+      <c r="S2" t="inlineStr">
         <is>
           <t>Anthodon panamense</t>
         </is>
       </c>
-      <c r="J2" t="inlineStr">
+      <c r="T2" t="inlineStr">
         <is>
           <t>Anthodon panamensis</t>
         </is>
       </c>
-      <c r="K2" t="inlineStr">
+      <c r="U2" t="inlineStr">
         <is>
           <t>A.C.Sm.</t>
         </is>
       </c>
-      <c r="L2" t="inlineStr">
-        <is>
-          <t>Species</t>
-        </is>
-      </c>
-      <c r="M2" t="inlineStr">
+      <c r="V2" t="inlineStr">
+        <is>
+          <t>Species</t>
+        </is>
+      </c>
+      <c r="W2" t="inlineStr">
         <is>
           <t>Synonym</t>
         </is>
       </c>
-      <c r="N2">
+      <c r="X2">
         <v>2641684</v>
       </c>
-      <c r="O2" t="inlineStr">
+      <c r="Y2" t="inlineStr">
         <is>
           <t>15016-2</t>
         </is>
       </c>
-      <c r="P2">
+      <c r="Z2">
         <v>0.895</v>
       </c>
-      <c r="Q2">
+      <c r="AA2">
         <v>2641675</v>
       </c>
-      <c r="R2" t="inlineStr">
+      <c r="AB2" t="inlineStr">
         <is>
           <t>430910-1</t>
         </is>
       </c>
-      <c r="S2" t="inlineStr">
+      <c r="AC2" t="inlineStr">
         <is>
           <t>430910-1</t>
         </is>
       </c>
-      <c r="T2" t="inlineStr">
+      <c r="AD2" t="inlineStr">
         <is>
           <t>Anthodon decussatum</t>
         </is>
       </c>
-      <c r="U2" t="inlineStr">
+      <c r="AE2" t="inlineStr">
         <is>
           <t>Anthodon</t>
         </is>
       </c>
-      <c r="V2" t="inlineStr">
+      <c r="AF2" t="inlineStr">
         <is>
           <t>decussatum</t>
         </is>
       </c>
-      <c r="W2" t="inlineStr">
-        <is>
-          <t>Species</t>
-        </is>
-      </c>
-      <c r="X2" t="inlineStr">
+      <c r="AG2" t="inlineStr">
+        <is>
+          <t>Species</t>
+        </is>
+      </c>
+      <c r="AH2" t="inlineStr">
         <is>
           <t>Celastraceae</t>
         </is>
       </c>
-      <c r="AA2" t="inlineStr">
+      <c r="AK2" t="inlineStr">
         <is>
           <t>Ruiz &amp; Pav.</t>
         </is>
       </c>
-      <c r="AB2" t="inlineStr">
+      <c r="AL2" t="inlineStr">
         <is>
           <t>Ruiz &amp; Pav.</t>
         </is>
       </c>
-      <c r="AC2" t="inlineStr">
+      <c r="AM2" t="inlineStr">
         <is>
           <t>liana</t>
         </is>
       </c>
-      <c r="AD2" t="b">
+      <c r="AN2" t="b">
         <v>0</v>
       </c>
     </row>
@@ -641,106 +709,106 @@
           <t>Blepharodon mucronatum</t>
         </is>
       </c>
-      <c r="D3" t="inlineStr">
+      <c r="G3" t="inlineStr">
         <is>
           <t>Blepharodon</t>
         </is>
       </c>
-      <c r="E3" t="inlineStr">
+      <c r="H3" t="inlineStr">
         <is>
           <t>mucronatum</t>
         </is>
       </c>
-      <c r="I3" t="inlineStr">
+      <c r="S3" t="inlineStr">
         <is>
           <t>Blepharodon mucronatum</t>
         </is>
       </c>
-      <c r="J3" t="inlineStr">
+      <c r="T3" t="inlineStr">
         <is>
           <t>Blepharodon mucronatum</t>
         </is>
       </c>
-      <c r="K3" t="inlineStr">
+      <c r="U3" t="inlineStr">
         <is>
           <t>(Schltdl.) Decne.</t>
         </is>
       </c>
-      <c r="L3" t="inlineStr">
-        <is>
-          <t>Species</t>
-        </is>
-      </c>
-      <c r="M3" t="inlineStr">
+      <c r="V3" t="inlineStr">
+        <is>
+          <t>Species</t>
+        </is>
+      </c>
+      <c r="W3" t="inlineStr">
         <is>
           <t>Synonym</t>
         </is>
       </c>
-      <c r="N3">
+      <c r="X3">
         <v>501746</v>
       </c>
-      <c r="O3" t="inlineStr">
+      <c r="Y3" t="inlineStr">
         <is>
           <t>94927-1</t>
         </is>
       </c>
-      <c r="P3">
-        <v>1</v>
-      </c>
-      <c r="Q3">
+      <c r="Z3">
+        <v>1</v>
+      </c>
+      <c r="AA3">
         <v>532478</v>
       </c>
-      <c r="R3" t="inlineStr">
+      <c r="AB3" t="inlineStr">
         <is>
           <t>60476540-2</t>
         </is>
       </c>
-      <c r="S3" t="inlineStr">
+      <c r="AC3" t="inlineStr">
         <is>
           <t>60476540-2</t>
         </is>
       </c>
-      <c r="T3" t="inlineStr">
+      <c r="AD3" t="inlineStr">
         <is>
           <t>Vailia anomala</t>
         </is>
       </c>
-      <c r="U3" t="inlineStr">
+      <c r="AE3" t="inlineStr">
         <is>
           <t>Vailia</t>
         </is>
       </c>
-      <c r="V3" t="inlineStr">
+      <c r="AF3" t="inlineStr">
         <is>
           <t>anomala</t>
         </is>
       </c>
-      <c r="W3" t="inlineStr">
-        <is>
-          <t>Species</t>
-        </is>
-      </c>
-      <c r="X3" t="inlineStr">
+      <c r="AG3" t="inlineStr">
+        <is>
+          <t>Species</t>
+        </is>
+      </c>
+      <c r="AH3" t="inlineStr">
         <is>
           <t>Apocynaceae</t>
         </is>
       </c>
-      <c r="AA3" t="inlineStr">
+      <c r="AK3" t="inlineStr">
         <is>
           <t>W.D.Stevens</t>
         </is>
       </c>
-      <c r="AB3" t="inlineStr">
+      <c r="AL3" t="inlineStr">
         <is>
           <t>(Brandegee) W.D.Stevens</t>
         </is>
       </c>
-      <c r="AC3" t="inlineStr">
+      <c r="AM3" t="inlineStr">
         <is>
           <t>subshrub</t>
         </is>
       </c>
-      <c r="AD3" t="b">
+      <c r="AN3" t="b">
         <v>1</v>
       </c>
     </row>
@@ -755,106 +823,106 @@
           <t>Cissus pseudosicyoides</t>
         </is>
       </c>
-      <c r="D4" t="inlineStr">
+      <c r="G4" t="inlineStr">
         <is>
           <t>Cissus</t>
         </is>
       </c>
-      <c r="E4" t="inlineStr">
+      <c r="H4" t="inlineStr">
         <is>
           <t>pseudosicyoides</t>
         </is>
       </c>
-      <c r="I4" t="inlineStr">
+      <c r="S4" t="inlineStr">
         <is>
           <t>Cissus pseudosicyoides</t>
         </is>
       </c>
-      <c r="J4" t="inlineStr">
+      <c r="T4" t="inlineStr">
         <is>
           <t>Cissus pseudosicyoides</t>
         </is>
       </c>
-      <c r="K4" t="inlineStr">
+      <c r="U4" t="inlineStr">
         <is>
           <t>Croat</t>
         </is>
       </c>
-      <c r="L4" t="inlineStr">
-        <is>
-          <t>Species</t>
-        </is>
-      </c>
-      <c r="M4" t="inlineStr">
+      <c r="V4" t="inlineStr">
+        <is>
+          <t>Species</t>
+        </is>
+      </c>
+      <c r="W4" t="inlineStr">
         <is>
           <t>Synonym</t>
         </is>
       </c>
-      <c r="N4">
+      <c r="X4">
         <v>2722815</v>
       </c>
-      <c r="O4" t="inlineStr">
+      <c r="Y4" t="inlineStr">
         <is>
           <t>59338-2</t>
         </is>
       </c>
-      <c r="P4">
-        <v>1</v>
-      </c>
-      <c r="Q4">
+      <c r="Z4">
+        <v>1</v>
+      </c>
+      <c r="AA4">
         <v>2722433</v>
       </c>
-      <c r="R4" t="inlineStr">
+      <c r="AB4" t="inlineStr">
         <is>
           <t>67664-1</t>
         </is>
       </c>
-      <c r="S4" t="inlineStr">
+      <c r="AC4" t="inlineStr">
         <is>
           <t>67664-1</t>
         </is>
       </c>
-      <c r="T4" t="inlineStr">
+      <c r="AD4" t="inlineStr">
         <is>
           <t>Cissus fuliginea</t>
         </is>
       </c>
-      <c r="U4" t="inlineStr">
+      <c r="AE4" t="inlineStr">
         <is>
           <t>Cissus</t>
         </is>
       </c>
-      <c r="V4" t="inlineStr">
+      <c r="AF4" t="inlineStr">
         <is>
           <t>fuliginea</t>
         </is>
       </c>
-      <c r="W4" t="inlineStr">
-        <is>
-          <t>Species</t>
-        </is>
-      </c>
-      <c r="X4" t="inlineStr">
+      <c r="AG4" t="inlineStr">
+        <is>
+          <t>Species</t>
+        </is>
+      </c>
+      <c r="AH4" t="inlineStr">
         <is>
           <t>Vitaceae</t>
         </is>
       </c>
-      <c r="AA4" t="inlineStr">
+      <c r="AK4" t="inlineStr">
         <is>
           <t>Kunth</t>
         </is>
       </c>
-      <c r="AB4" t="inlineStr">
+      <c r="AL4" t="inlineStr">
         <is>
           <t>Kunth</t>
         </is>
       </c>
-      <c r="AC4" t="inlineStr">
+      <c r="AM4" t="inlineStr">
         <is>
           <t>climber</t>
         </is>
       </c>
-      <c r="AD4" t="b">
+      <c r="AN4" t="b">
         <v>1</v>
       </c>
     </row>
@@ -869,106 +937,106 @@
           <t>Cissus rhombifolia</t>
         </is>
       </c>
-      <c r="D5" t="inlineStr">
+      <c r="G5" t="inlineStr">
         <is>
           <t>Cissus</t>
         </is>
       </c>
-      <c r="E5" t="inlineStr">
+      <c r="H5" t="inlineStr">
         <is>
           <t>rhombifolia</t>
         </is>
       </c>
-      <c r="I5" t="inlineStr">
+      <c r="S5" t="inlineStr">
         <is>
           <t>Cissus rhombifolia</t>
         </is>
       </c>
-      <c r="J5" t="inlineStr">
+      <c r="T5" t="inlineStr">
         <is>
           <t>Cissus rhombifolia</t>
         </is>
       </c>
-      <c r="K5" t="inlineStr">
+      <c r="U5" t="inlineStr">
         <is>
           <t>Vahl</t>
         </is>
       </c>
-      <c r="L5" t="inlineStr">
-        <is>
-          <t>Species</t>
-        </is>
-      </c>
-      <c r="M5" t="inlineStr">
+      <c r="V5" t="inlineStr">
+        <is>
+          <t>Species</t>
+        </is>
+      </c>
+      <c r="W5" t="inlineStr">
         <is>
           <t>Synonym</t>
         </is>
       </c>
-      <c r="N5">
+      <c r="X5">
         <v>2722860</v>
       </c>
-      <c r="O5" t="inlineStr">
+      <c r="Y5" t="inlineStr">
         <is>
           <t>301239-2</t>
         </is>
       </c>
-      <c r="P5">
-        <v>1</v>
-      </c>
-      <c r="Q5">
+      <c r="Z5">
+        <v>1</v>
+      </c>
+      <c r="AA5">
         <v>2722134</v>
       </c>
-      <c r="R5" t="inlineStr">
+      <c r="AB5" t="inlineStr">
         <is>
           <t>311226-2</t>
         </is>
       </c>
-      <c r="S5" t="inlineStr">
+      <c r="AC5" t="inlineStr">
         <is>
           <t>311226-2</t>
         </is>
       </c>
-      <c r="T5" t="inlineStr">
+      <c r="AD5" t="inlineStr">
         <is>
           <t>Cissus alata</t>
         </is>
       </c>
-      <c r="U5" t="inlineStr">
+      <c r="AE5" t="inlineStr">
         <is>
           <t>Cissus</t>
         </is>
       </c>
-      <c r="V5" t="inlineStr">
+      <c r="AF5" t="inlineStr">
         <is>
           <t>alata</t>
         </is>
       </c>
-      <c r="W5" t="inlineStr">
-        <is>
-          <t>Species</t>
-        </is>
-      </c>
-      <c r="X5" t="inlineStr">
+      <c r="AG5" t="inlineStr">
+        <is>
+          <t>Species</t>
+        </is>
+      </c>
+      <c r="AH5" t="inlineStr">
         <is>
           <t>Vitaceae</t>
         </is>
       </c>
-      <c r="AA5" t="inlineStr">
+      <c r="AK5" t="inlineStr">
         <is>
           <t>Jacq.</t>
         </is>
       </c>
-      <c r="AB5" t="inlineStr">
+      <c r="AL5" t="inlineStr">
         <is>
           <t>Jacq.</t>
         </is>
       </c>
-      <c r="AC5" t="inlineStr">
+      <c r="AM5" t="inlineStr">
         <is>
           <t>liana</t>
         </is>
       </c>
-      <c r="AD5" t="b">
+      <c r="AN5" t="b">
         <v>1</v>
       </c>
     </row>
@@ -983,106 +1051,106 @@
           <t>Cissus sicyoides</t>
         </is>
       </c>
-      <c r="D6" t="inlineStr">
+      <c r="G6" t="inlineStr">
         <is>
           <t>Cissus</t>
         </is>
       </c>
-      <c r="E6" t="inlineStr">
+      <c r="H6" t="inlineStr">
         <is>
           <t>sicyoides</t>
         </is>
       </c>
-      <c r="I6" t="inlineStr">
+      <c r="S6" t="inlineStr">
         <is>
           <t>Cissus sicyoides</t>
         </is>
       </c>
-      <c r="J6" t="inlineStr">
+      <c r="T6" t="inlineStr">
         <is>
           <t>Cissus sicyoides</t>
         </is>
       </c>
-      <c r="K6" t="inlineStr">
+      <c r="U6" t="inlineStr">
         <is>
           <t>L.</t>
         </is>
       </c>
-      <c r="L6" t="inlineStr">
-        <is>
-          <t>Species</t>
-        </is>
-      </c>
-      <c r="M6" t="inlineStr">
+      <c r="V6" t="inlineStr">
+        <is>
+          <t>Species</t>
+        </is>
+      </c>
+      <c r="W6" t="inlineStr">
         <is>
           <t>Synonym</t>
         </is>
       </c>
-      <c r="N6">
+      <c r="X6">
         <v>2722937</v>
       </c>
-      <c r="O6" t="inlineStr">
+      <c r="Y6" t="inlineStr">
         <is>
           <t>67960-1</t>
         </is>
       </c>
-      <c r="P6">
-        <v>1</v>
-      </c>
-      <c r="Q6">
+      <c r="Z6">
+        <v>1</v>
+      </c>
+      <c r="AA6">
         <v>3262817</v>
       </c>
-      <c r="R6" t="inlineStr">
+      <c r="AB6" t="inlineStr">
         <is>
           <t>77228002-1</t>
         </is>
       </c>
-      <c r="S6" t="inlineStr">
+      <c r="AC6" t="inlineStr">
         <is>
           <t>77228002-1</t>
         </is>
       </c>
-      <c r="T6" t="inlineStr">
+      <c r="AD6" t="inlineStr">
         <is>
           <t>Cissus verticillata subsp. verticillata</t>
         </is>
       </c>
-      <c r="U6" t="inlineStr">
+      <c r="AE6" t="inlineStr">
         <is>
           <t>Cissus</t>
         </is>
       </c>
-      <c r="V6" t="inlineStr">
+      <c r="AF6" t="inlineStr">
         <is>
           <t>verticillata</t>
         </is>
       </c>
-      <c r="W6" t="inlineStr">
+      <c r="AG6" t="inlineStr">
         <is>
           <t>Subspecies</t>
         </is>
       </c>
-      <c r="X6" t="inlineStr">
+      <c r="AH6" t="inlineStr">
         <is>
           <t>Vitaceae</t>
         </is>
       </c>
-      <c r="Y6" t="inlineStr">
+      <c r="AI6" t="inlineStr">
         <is>
           <t>subsp.</t>
         </is>
       </c>
-      <c r="Z6" t="inlineStr">
+      <c r="AJ6" t="inlineStr">
         <is>
           <t>verticillata</t>
         </is>
       </c>
-      <c r="AC6" t="inlineStr">
+      <c r="AM6" t="inlineStr">
         <is>
           <t>liana</t>
         </is>
       </c>
-      <c r="AD6" t="b">
+      <c r="AN6" t="b">
         <v>1</v>
       </c>
     </row>
@@ -1097,106 +1165,106 @@
           <t>Clitoria rubiginosa</t>
         </is>
       </c>
-      <c r="D7" t="inlineStr">
+      <c r="G7" t="inlineStr">
         <is>
           <t>Clitoria</t>
         </is>
       </c>
-      <c r="E7" t="inlineStr">
+      <c r="H7" t="inlineStr">
         <is>
           <t>rubiginosa</t>
         </is>
       </c>
-      <c r="I7" t="inlineStr">
+      <c r="S7" t="inlineStr">
         <is>
           <t>Clitoria rubiginosa</t>
         </is>
       </c>
-      <c r="J7" t="inlineStr">
+      <c r="T7" t="inlineStr">
         <is>
           <t>Clitoria rubiginosa</t>
         </is>
       </c>
-      <c r="K7" t="inlineStr">
+      <c r="U7" t="inlineStr">
         <is>
           <t>Juss. ex Pers.</t>
         </is>
       </c>
-      <c r="L7" t="inlineStr">
-        <is>
-          <t>Species</t>
-        </is>
-      </c>
-      <c r="M7" t="inlineStr">
+      <c r="V7" t="inlineStr">
+        <is>
+          <t>Species</t>
+        </is>
+      </c>
+      <c r="W7" t="inlineStr">
         <is>
           <t>Synonym</t>
         </is>
       </c>
-      <c r="N7">
+      <c r="X7">
         <v>2728091</v>
       </c>
-      <c r="O7" t="inlineStr">
+      <c r="Y7" t="inlineStr">
         <is>
           <t>486592-1</t>
         </is>
       </c>
-      <c r="P7">
-        <v>1</v>
-      </c>
-      <c r="Q7">
+      <c r="Z7">
+        <v>1</v>
+      </c>
+      <c r="AA7">
         <v>3256130</v>
       </c>
-      <c r="R7" t="inlineStr">
+      <c r="AB7" t="inlineStr">
         <is>
           <t>77223719-1</t>
         </is>
       </c>
-      <c r="S7" t="inlineStr">
+      <c r="AC7" t="inlineStr">
         <is>
           <t>77223719-1</t>
         </is>
       </c>
-      <c r="T7" t="inlineStr">
+      <c r="AD7" t="inlineStr">
         <is>
           <t>Clitoria falcata var. falcata</t>
         </is>
       </c>
-      <c r="U7" t="inlineStr">
+      <c r="AE7" t="inlineStr">
         <is>
           <t>Clitoria</t>
         </is>
       </c>
-      <c r="V7" t="inlineStr">
+      <c r="AF7" t="inlineStr">
         <is>
           <t>falcata</t>
         </is>
       </c>
-      <c r="W7" t="inlineStr">
+      <c r="AG7" t="inlineStr">
         <is>
           <t>Variety</t>
         </is>
       </c>
-      <c r="X7" t="inlineStr">
+      <c r="AH7" t="inlineStr">
         <is>
           <t>Fabaceae</t>
         </is>
       </c>
-      <c r="Y7" t="inlineStr">
+      <c r="AI7" t="inlineStr">
         <is>
           <t>var.</t>
         </is>
       </c>
-      <c r="Z7" t="inlineStr">
+      <c r="AJ7" t="inlineStr">
         <is>
           <t>falcata</t>
         </is>
       </c>
-      <c r="AC7" t="inlineStr">
+      <c r="AM7" t="inlineStr">
         <is>
           <t>climbing perennial</t>
         </is>
       </c>
-      <c r="AD7" t="b">
+      <c r="AN7" t="b">
         <v>1</v>
       </c>
     </row>
@@ -1211,106 +1279,106 @@
           <t>Clytostoma binatum</t>
         </is>
       </c>
-      <c r="D8" t="inlineStr">
+      <c r="G8" t="inlineStr">
         <is>
           <t>Clytostoma</t>
         </is>
       </c>
-      <c r="E8" t="inlineStr">
+      <c r="H8" t="inlineStr">
         <is>
           <t>binatum</t>
         </is>
       </c>
-      <c r="I8" t="inlineStr">
+      <c r="S8" t="inlineStr">
         <is>
           <t>Clytostoma binatum</t>
         </is>
       </c>
-      <c r="J8" t="inlineStr">
+      <c r="T8" t="inlineStr">
         <is>
           <t>Clytostoma binatum</t>
         </is>
       </c>
-      <c r="K8" t="inlineStr">
+      <c r="U8" t="inlineStr">
         <is>
           <t>(Thunb.) Sandwith</t>
         </is>
       </c>
-      <c r="L8" t="inlineStr">
-        <is>
-          <t>Species</t>
-        </is>
-      </c>
-      <c r="M8" t="inlineStr">
+      <c r="V8" t="inlineStr">
+        <is>
+          <t>Species</t>
+        </is>
+      </c>
+      <c r="W8" t="inlineStr">
         <is>
           <t>Synonym</t>
         </is>
       </c>
-      <c r="N8">
+      <c r="X8">
         <v>320873</v>
       </c>
-      <c r="O8" t="inlineStr">
+      <c r="Y8" t="inlineStr">
         <is>
           <t>61651-2</t>
         </is>
       </c>
-      <c r="P8">
-        <v>1</v>
-      </c>
-      <c r="Q8">
+      <c r="Z8">
+        <v>1</v>
+      </c>
+      <c r="AA8">
         <v>319839</v>
       </c>
-      <c r="R8" t="inlineStr">
+      <c r="AB8" t="inlineStr">
         <is>
           <t>108602-1</t>
         </is>
       </c>
-      <c r="S8" t="inlineStr">
+      <c r="AC8" t="inlineStr">
         <is>
           <t>108602-1</t>
         </is>
       </c>
-      <c r="T8" t="inlineStr">
+      <c r="AD8" t="inlineStr">
         <is>
           <t>Bignonia binata</t>
         </is>
       </c>
-      <c r="U8" t="inlineStr">
+      <c r="AE8" t="inlineStr">
         <is>
           <t>Bignonia</t>
         </is>
       </c>
-      <c r="V8" t="inlineStr">
+      <c r="AF8" t="inlineStr">
         <is>
           <t>binata</t>
         </is>
       </c>
-      <c r="W8" t="inlineStr">
-        <is>
-          <t>Species</t>
-        </is>
-      </c>
-      <c r="X8" t="inlineStr">
+      <c r="AG8" t="inlineStr">
+        <is>
+          <t>Species</t>
+        </is>
+      </c>
+      <c r="AH8" t="inlineStr">
         <is>
           <t>Bignoniaceae</t>
         </is>
       </c>
-      <c r="AA8" t="inlineStr">
+      <c r="AK8" t="inlineStr">
         <is>
           <t>Thunb.</t>
         </is>
       </c>
-      <c r="AB8" t="inlineStr">
+      <c r="AL8" t="inlineStr">
         <is>
           <t>Thunb.</t>
         </is>
       </c>
-      <c r="AC8" t="inlineStr">
+      <c r="AM8" t="inlineStr">
         <is>
           <t>liana</t>
         </is>
       </c>
-      <c r="AD8" t="b">
+      <c r="AN8" t="b">
         <v>1</v>
       </c>
     </row>
@@ -1327,114 +1395,132 @@
       </c>
       <c r="C9" t="inlineStr">
         <is>
+          <t>NA NA</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>Cydista aequinoctialis</t>
+        </is>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>NA NA</t>
+        </is>
+      </c>
+      <c r="F9" t="inlineStr">
+        <is>
           <t>Bignoniaceae</t>
         </is>
       </c>
-      <c r="D9" t="inlineStr">
+      <c r="G9" t="inlineStr">
         <is>
           <t>Cydista</t>
         </is>
       </c>
-      <c r="E9" t="inlineStr">
+      <c r="H9" t="inlineStr">
         <is>
           <t>aequinoctialis</t>
         </is>
       </c>
-      <c r="F9" t="inlineStr">
+      <c r="J9" t="inlineStr">
         <is>
           <t>(L.) Miers</t>
         </is>
       </c>
-      <c r="I9" t="inlineStr">
+      <c r="P9" t="b">
+        <v>1</v>
+      </c>
+      <c r="S9" t="inlineStr">
         <is>
           <t>Cydista aequinoctialis</t>
         </is>
       </c>
-      <c r="J9" t="inlineStr">
+      <c r="T9" t="inlineStr">
         <is>
           <t>Cydista aequinoctialis</t>
         </is>
       </c>
-      <c r="K9" t="inlineStr">
+      <c r="U9" t="inlineStr">
         <is>
           <t>(L.) Miers</t>
         </is>
       </c>
-      <c r="L9" t="inlineStr">
-        <is>
-          <t>Species</t>
-        </is>
-      </c>
-      <c r="M9" t="inlineStr">
+      <c r="V9" t="inlineStr">
+        <is>
+          <t>Species</t>
+        </is>
+      </c>
+      <c r="W9" t="inlineStr">
         <is>
           <t>Synonym</t>
         </is>
       </c>
-      <c r="N9">
+      <c r="X9">
         <v>320596</v>
       </c>
-      <c r="O9" t="inlineStr">
+      <c r="Y9" t="inlineStr">
         <is>
           <t>109402-1</t>
         </is>
       </c>
-      <c r="P9">
-        <v>1</v>
-      </c>
-      <c r="Q9">
+      <c r="Z9">
+        <v>1</v>
+      </c>
+      <c r="AA9">
         <v>319795</v>
       </c>
-      <c r="R9" t="inlineStr">
+      <c r="AB9" t="inlineStr">
         <is>
           <t>108550-1</t>
         </is>
       </c>
-      <c r="S9" t="inlineStr">
+      <c r="AC9" t="inlineStr">
         <is>
           <t>108550-1</t>
         </is>
       </c>
-      <c r="T9" t="inlineStr">
+      <c r="AD9" t="inlineStr">
         <is>
           <t>Bignonia aequinoctialis</t>
         </is>
       </c>
-      <c r="U9" t="inlineStr">
+      <c r="AE9" t="inlineStr">
         <is>
           <t>Bignonia</t>
         </is>
       </c>
-      <c r="V9" t="inlineStr">
+      <c r="AF9" t="inlineStr">
         <is>
           <t>aequinoctialis</t>
         </is>
       </c>
-      <c r="W9" t="inlineStr">
-        <is>
-          <t>Species</t>
-        </is>
-      </c>
-      <c r="X9" t="inlineStr">
+      <c r="AG9" t="inlineStr">
+        <is>
+          <t>Species</t>
+        </is>
+      </c>
+      <c r="AH9" t="inlineStr">
         <is>
           <t>Bignoniaceae</t>
         </is>
       </c>
-      <c r="AA9" t="inlineStr">
+      <c r="AK9" t="inlineStr">
         <is>
           <t>L.</t>
         </is>
       </c>
-      <c r="AB9" t="inlineStr">
+      <c r="AL9" t="inlineStr">
         <is>
           <t>L.</t>
         </is>
       </c>
-      <c r="AC9" t="inlineStr">
+      <c r="AM9" t="inlineStr">
         <is>
           <t>liana</t>
         </is>
       </c>
-      <c r="AD9" t="b">
+      <c r="AN9" t="b">
         <v>1</v>
       </c>
     </row>
@@ -1449,106 +1535,106 @@
           <t>Forsteronia peninsularis</t>
         </is>
       </c>
-      <c r="D10" t="inlineStr">
+      <c r="G10" t="inlineStr">
         <is>
           <t>Forsteronia</t>
         </is>
       </c>
-      <c r="E10" t="inlineStr">
+      <c r="H10" t="inlineStr">
         <is>
           <t>peninsularis</t>
         </is>
       </c>
-      <c r="I10" t="inlineStr">
+      <c r="S10" t="inlineStr">
         <is>
           <t>Forsteronia peninsularis</t>
         </is>
       </c>
-      <c r="J10" t="inlineStr">
+      <c r="T10" t="inlineStr">
         <is>
           <t>Forsteronia peninsularis</t>
         </is>
       </c>
-      <c r="K10" t="inlineStr">
+      <c r="U10" t="inlineStr">
         <is>
           <t>Woodson</t>
         </is>
       </c>
-      <c r="L10" t="inlineStr">
-        <is>
-          <t>Species</t>
-        </is>
-      </c>
-      <c r="M10" t="inlineStr">
+      <c r="V10" t="inlineStr">
+        <is>
+          <t>Species</t>
+        </is>
+      </c>
+      <c r="W10" t="inlineStr">
         <is>
           <t>Synonym</t>
         </is>
       </c>
-      <c r="N10">
+      <c r="X10">
         <v>84743</v>
       </c>
-      <c r="O10" t="inlineStr">
+      <c r="Y10" t="inlineStr">
         <is>
           <t>105377-2</t>
         </is>
       </c>
-      <c r="P10">
-        <v>1</v>
-      </c>
-      <c r="Q10">
+      <c r="Z10">
+        <v>1</v>
+      </c>
+      <c r="AA10">
         <v>347877</v>
       </c>
-      <c r="R10" t="inlineStr">
+      <c r="AB10" t="inlineStr">
         <is>
           <t>77084117-1</t>
         </is>
       </c>
-      <c r="S10" t="inlineStr">
+      <c r="AC10" t="inlineStr">
         <is>
           <t>77084117-1</t>
         </is>
       </c>
-      <c r="T10" t="inlineStr">
+      <c r="AD10" t="inlineStr">
         <is>
           <t>Pinochia peninsularis</t>
         </is>
       </c>
-      <c r="U10" t="inlineStr">
+      <c r="AE10" t="inlineStr">
         <is>
           <t>Pinochia</t>
         </is>
       </c>
-      <c r="V10" t="inlineStr">
+      <c r="AF10" t="inlineStr">
         <is>
           <t>peninsularis</t>
         </is>
       </c>
-      <c r="W10" t="inlineStr">
-        <is>
-          <t>Species</t>
-        </is>
-      </c>
-      <c r="X10" t="inlineStr">
+      <c r="AG10" t="inlineStr">
+        <is>
+          <t>Species</t>
+        </is>
+      </c>
+      <c r="AH10" t="inlineStr">
         <is>
           <t>Apocynaceae</t>
         </is>
       </c>
-      <c r="AA10" t="inlineStr">
+      <c r="AK10" t="inlineStr">
         <is>
           <t>M.E.Endress &amp; B.F.Hansen</t>
         </is>
       </c>
-      <c r="AB10" t="inlineStr">
+      <c r="AL10" t="inlineStr">
         <is>
           <t>(Woodson) M.E.Endress &amp; B.F.Hansen</t>
         </is>
       </c>
-      <c r="AC10" t="inlineStr">
+      <c r="AM10" t="inlineStr">
         <is>
           <t>climber</t>
         </is>
       </c>
-      <c r="AD10" t="b">
+      <c r="AN10" t="b">
         <v>1</v>
       </c>
     </row>
@@ -1563,106 +1649,106 @@
           <t>Gouania adenophera</t>
         </is>
       </c>
-      <c r="D11" t="inlineStr">
+      <c r="G11" t="inlineStr">
         <is>
           <t>Gouania</t>
         </is>
       </c>
-      <c r="E11" t="inlineStr">
+      <c r="H11" t="inlineStr">
         <is>
           <t>adenophera</t>
         </is>
       </c>
-      <c r="I11" t="inlineStr">
+      <c r="S11" t="inlineStr">
         <is>
           <t>Gouania adenophera</t>
         </is>
       </c>
-      <c r="J11" t="inlineStr">
+      <c r="T11" t="inlineStr">
         <is>
           <t>Gouania adenophora</t>
         </is>
       </c>
-      <c r="K11" t="inlineStr">
+      <c r="U11" t="inlineStr">
         <is>
           <t>Pilg.</t>
         </is>
       </c>
-      <c r="L11" t="inlineStr">
-        <is>
-          <t>Species</t>
-        </is>
-      </c>
-      <c r="M11" t="inlineStr">
+      <c r="V11" t="inlineStr">
+        <is>
+          <t>Species</t>
+        </is>
+      </c>
+      <c r="W11" t="inlineStr">
         <is>
           <t>Synonym</t>
         </is>
       </c>
-      <c r="N11">
+      <c r="X11">
         <v>2831381</v>
       </c>
-      <c r="O11" t="inlineStr">
+      <c r="Y11" t="inlineStr">
         <is>
           <t>112849-2</t>
         </is>
       </c>
-      <c r="P11">
+      <c r="Z11">
         <v>0.944</v>
       </c>
-      <c r="Q11">
+      <c r="AA11">
         <v>2831420</v>
       </c>
-      <c r="R11" t="inlineStr">
+      <c r="AB11" t="inlineStr">
         <is>
           <t>717458-1</t>
         </is>
       </c>
-      <c r="S11" t="inlineStr">
+      <c r="AC11" t="inlineStr">
         <is>
           <t>717458-1</t>
         </is>
       </c>
-      <c r="T11" t="inlineStr">
+      <c r="AD11" t="inlineStr">
         <is>
           <t>Gouania frangulifolia</t>
         </is>
       </c>
-      <c r="U11" t="inlineStr">
+      <c r="AE11" t="inlineStr">
         <is>
           <t>Gouania</t>
         </is>
       </c>
-      <c r="V11" t="inlineStr">
+      <c r="AF11" t="inlineStr">
         <is>
           <t>frangulifolia</t>
         </is>
       </c>
-      <c r="W11" t="inlineStr">
-        <is>
-          <t>Species</t>
-        </is>
-      </c>
-      <c r="X11" t="inlineStr">
+      <c r="AG11" t="inlineStr">
+        <is>
+          <t>Species</t>
+        </is>
+      </c>
+      <c r="AH11" t="inlineStr">
         <is>
           <t>Rhamnaceae</t>
         </is>
       </c>
-      <c r="AA11" t="inlineStr">
+      <c r="AK11" t="inlineStr">
         <is>
           <t>Radlk.</t>
         </is>
       </c>
-      <c r="AB11" t="inlineStr">
+      <c r="AL11" t="inlineStr">
         <is>
           <t>Radlk.</t>
         </is>
       </c>
-      <c r="AC11" t="inlineStr">
+      <c r="AM11" t="inlineStr">
         <is>
           <t>climber</t>
         </is>
       </c>
-      <c r="AD11" t="b">
+      <c r="AN11" t="b">
         <v>0</v>
       </c>
     </row>
@@ -1677,106 +1763,106 @@
           <t>Gurania coccinea</t>
         </is>
       </c>
-      <c r="D12" t="inlineStr">
+      <c r="G12" t="inlineStr">
         <is>
           <t>Gurania</t>
         </is>
       </c>
-      <c r="E12" t="inlineStr">
+      <c r="H12" t="inlineStr">
         <is>
           <t>coccinea</t>
         </is>
       </c>
-      <c r="I12" t="inlineStr">
+      <c r="S12" t="inlineStr">
         <is>
           <t>Gurania coccinea</t>
         </is>
       </c>
-      <c r="J12" t="inlineStr">
+      <c r="T12" t="inlineStr">
         <is>
           <t>Gurania coccinea</t>
         </is>
       </c>
-      <c r="K12" t="inlineStr">
+      <c r="U12" t="inlineStr">
         <is>
           <t>Cogn.</t>
         </is>
       </c>
-      <c r="L12" t="inlineStr">
-        <is>
-          <t>Species</t>
-        </is>
-      </c>
-      <c r="M12" t="inlineStr">
+      <c r="V12" t="inlineStr">
+        <is>
+          <t>Species</t>
+        </is>
+      </c>
+      <c r="W12" t="inlineStr">
         <is>
           <t>Synonym</t>
         </is>
       </c>
-      <c r="N12">
+      <c r="X12">
         <v>2835145</v>
       </c>
-      <c r="O12" t="inlineStr">
+      <c r="Y12" t="inlineStr">
         <is>
           <t>292778-1</t>
         </is>
       </c>
-      <c r="P12">
-        <v>1</v>
-      </c>
-      <c r="Q12">
+      <c r="Z12">
+        <v>1</v>
+      </c>
+      <c r="AA12">
         <v>2835132</v>
       </c>
-      <c r="R12" t="inlineStr">
+      <c r="AB12" t="inlineStr">
         <is>
           <t>114819-2</t>
         </is>
       </c>
-      <c r="S12" t="inlineStr">
+      <c r="AC12" t="inlineStr">
         <is>
           <t>114819-2</t>
         </is>
       </c>
-      <c r="T12" t="inlineStr">
+      <c r="AD12" t="inlineStr">
         <is>
           <t>Gurania bignoniacea</t>
         </is>
       </c>
-      <c r="U12" t="inlineStr">
+      <c r="AE12" t="inlineStr">
         <is>
           <t>Gurania</t>
         </is>
       </c>
-      <c r="V12" t="inlineStr">
+      <c r="AF12" t="inlineStr">
         <is>
           <t>bignoniacea</t>
         </is>
       </c>
-      <c r="W12" t="inlineStr">
-        <is>
-          <t>Species</t>
-        </is>
-      </c>
-      <c r="X12" t="inlineStr">
+      <c r="AG12" t="inlineStr">
+        <is>
+          <t>Species</t>
+        </is>
+      </c>
+      <c r="AH12" t="inlineStr">
         <is>
           <t>Cucurbitaceae</t>
         </is>
       </c>
-      <c r="AA12" t="inlineStr">
+      <c r="AK12" t="inlineStr">
         <is>
           <t>C.Jeffrey</t>
         </is>
       </c>
-      <c r="AB12" t="inlineStr">
+      <c r="AL12" t="inlineStr">
         <is>
           <t>(Poepp. &amp; Endl.) C.Jeffrey</t>
         </is>
       </c>
-      <c r="AC12" t="inlineStr">
+      <c r="AM12" t="inlineStr">
         <is>
           <t>climber</t>
         </is>
       </c>
-      <c r="AD12" t="b">
+      <c r="AN12" t="b">
         <v>1</v>
       </c>
     </row>
@@ -1793,114 +1879,132 @@
       </c>
       <c r="C13" t="inlineStr">
         <is>
+          <t>NA NA</t>
+        </is>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>Ipomoea phillomega</t>
+        </is>
+      </c>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t>NA NA</t>
+        </is>
+      </c>
+      <c r="F13" t="inlineStr">
+        <is>
           <t>Convolvulaceae</t>
         </is>
       </c>
-      <c r="D13" t="inlineStr">
+      <c r="G13" t="inlineStr">
         <is>
           <t>Ipomoea</t>
         </is>
       </c>
-      <c r="E13" t="inlineStr">
+      <c r="H13" t="inlineStr">
         <is>
           <t>phillomega</t>
         </is>
       </c>
-      <c r="F13" t="inlineStr">
+      <c r="J13" t="inlineStr">
         <is>
           <t>(Vell.) Casa</t>
         </is>
       </c>
-      <c r="I13" t="inlineStr">
+      <c r="P13" t="b">
+        <v>1</v>
+      </c>
+      <c r="S13" t="inlineStr">
         <is>
           <t>Ipomoea phillomega</t>
         </is>
       </c>
-      <c r="J13" t="inlineStr">
+      <c r="T13" t="inlineStr">
         <is>
           <t>Ipomoea philomega</t>
         </is>
       </c>
-      <c r="K13" t="inlineStr">
+      <c r="U13" t="inlineStr">
         <is>
           <t>(Vell.) House</t>
         </is>
       </c>
-      <c r="L13" t="inlineStr">
-        <is>
-          <t>Species</t>
-        </is>
-      </c>
-      <c r="M13" t="inlineStr">
+      <c r="V13" t="inlineStr">
+        <is>
+          <t>Species</t>
+        </is>
+      </c>
+      <c r="W13" t="inlineStr">
         <is>
           <t>Accepted</t>
         </is>
       </c>
-      <c r="N13">
+      <c r="X13">
         <v>480356</v>
       </c>
-      <c r="O13" t="inlineStr">
+      <c r="Y13" t="inlineStr">
         <is>
           <t>129579-2</t>
         </is>
       </c>
-      <c r="P13">
+      <c r="Z13">
         <v>0.944</v>
       </c>
-      <c r="Q13">
+      <c r="AA13">
         <v>480356</v>
       </c>
-      <c r="R13" t="inlineStr">
+      <c r="AB13" t="inlineStr">
         <is>
           <t>129579-2</t>
         </is>
       </c>
-      <c r="S13" t="inlineStr">
+      <c r="AC13" t="inlineStr">
         <is>
           <t>129579-2</t>
         </is>
       </c>
-      <c r="T13" t="inlineStr">
+      <c r="AD13" t="inlineStr">
         <is>
           <t>Ipomoea philomega</t>
         </is>
       </c>
-      <c r="U13" t="inlineStr">
+      <c r="AE13" t="inlineStr">
         <is>
           <t>Ipomoea</t>
         </is>
       </c>
-      <c r="V13" t="inlineStr">
+      <c r="AF13" t="inlineStr">
         <is>
           <t>philomega</t>
         </is>
       </c>
-      <c r="W13" t="inlineStr">
-        <is>
-          <t>Species</t>
-        </is>
-      </c>
-      <c r="X13" t="inlineStr">
+      <c r="AG13" t="inlineStr">
+        <is>
+          <t>Species</t>
+        </is>
+      </c>
+      <c r="AH13" t="inlineStr">
         <is>
           <t>Convolvulaceae</t>
         </is>
       </c>
-      <c r="AA13" t="inlineStr">
+      <c r="AK13" t="inlineStr">
         <is>
           <t>House</t>
         </is>
       </c>
-      <c r="AB13" t="inlineStr">
+      <c r="AL13" t="inlineStr">
         <is>
           <t>(Vell.) House</t>
         </is>
       </c>
-      <c r="AC13" t="inlineStr">
+      <c r="AM13" t="inlineStr">
         <is>
           <t>liana</t>
         </is>
       </c>
-      <c r="AD13" t="b">
+      <c r="AN13" t="b">
         <v>0</v>
       </c>
     </row>
@@ -1915,106 +2019,106 @@
           <t>Markea ulei</t>
         </is>
       </c>
-      <c r="D14" t="inlineStr">
+      <c r="G14" t="inlineStr">
         <is>
           <t>Markea</t>
         </is>
       </c>
-      <c r="E14" t="inlineStr">
+      <c r="H14" t="inlineStr">
         <is>
           <t>ulei</t>
         </is>
       </c>
-      <c r="I14" t="inlineStr">
+      <c r="S14" t="inlineStr">
         <is>
           <t>Markea ulei</t>
         </is>
       </c>
-      <c r="J14" t="inlineStr">
+      <c r="T14" t="inlineStr">
         <is>
           <t>Markea ulei</t>
         </is>
       </c>
-      <c r="K14" t="inlineStr">
+      <c r="U14" t="inlineStr">
         <is>
           <t>(Dammer) Cuatrec.</t>
         </is>
       </c>
-      <c r="L14" t="inlineStr">
-        <is>
-          <t>Species</t>
-        </is>
-      </c>
-      <c r="M14" t="inlineStr">
+      <c r="V14" t="inlineStr">
+        <is>
+          <t>Species</t>
+        </is>
+      </c>
+      <c r="W14" t="inlineStr">
         <is>
           <t>Synonym</t>
         </is>
       </c>
-      <c r="N14">
+      <c r="X14">
         <v>2508288</v>
       </c>
-      <c r="O14" t="inlineStr">
+      <c r="Y14" t="inlineStr">
         <is>
           <t>153428-2</t>
         </is>
       </c>
-      <c r="P14">
-        <v>1</v>
-      </c>
-      <c r="Q14">
+      <c r="Z14">
+        <v>1</v>
+      </c>
+      <c r="AA14">
         <v>2840332</v>
       </c>
-      <c r="R14" t="inlineStr">
+      <c r="AB14" t="inlineStr">
         <is>
           <t>118130-2</t>
         </is>
       </c>
-      <c r="S14" t="inlineStr">
+      <c r="AC14" t="inlineStr">
         <is>
           <t>118130-2</t>
         </is>
       </c>
-      <c r="T14" t="inlineStr">
+      <c r="AD14" t="inlineStr">
         <is>
           <t>Hawkesiophyton ulei</t>
         </is>
       </c>
-      <c r="U14" t="inlineStr">
+      <c r="AE14" t="inlineStr">
         <is>
           <t>Hawkesiophyton</t>
         </is>
       </c>
-      <c r="V14" t="inlineStr">
+      <c r="AF14" t="inlineStr">
         <is>
           <t>ulei</t>
         </is>
       </c>
-      <c r="W14" t="inlineStr">
-        <is>
-          <t>Species</t>
-        </is>
-      </c>
-      <c r="X14" t="inlineStr">
+      <c r="AG14" t="inlineStr">
+        <is>
+          <t>Species</t>
+        </is>
+      </c>
+      <c r="AH14" t="inlineStr">
         <is>
           <t>Solanaceae</t>
         </is>
       </c>
-      <c r="AA14" t="inlineStr">
+      <c r="AK14" t="inlineStr">
         <is>
           <t>Hunz.</t>
         </is>
       </c>
-      <c r="AB14" t="inlineStr">
+      <c r="AL14" t="inlineStr">
         <is>
           <t>(Dammer) Hunz.</t>
         </is>
       </c>
-      <c r="AC14" t="inlineStr">
+      <c r="AM14" t="inlineStr">
         <is>
           <t>climbing epiphyte</t>
         </is>
       </c>
-      <c r="AD14" t="b">
+      <c r="AN14" t="b">
         <v>1</v>
       </c>
     </row>
@@ -2031,114 +2135,132 @@
       </c>
       <c r="C15" t="inlineStr">
         <is>
+          <t>NA NA</t>
+        </is>
+      </c>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t>Marsdenia crassipes</t>
+        </is>
+      </c>
+      <c r="E15" t="inlineStr">
+        <is>
+          <t>NA NA</t>
+        </is>
+      </c>
+      <c r="F15" t="inlineStr">
+        <is>
           <t>Asclepiadaceae</t>
         </is>
       </c>
-      <c r="D15" t="inlineStr">
+      <c r="G15" t="inlineStr">
         <is>
           <t>Marsdenia</t>
         </is>
       </c>
-      <c r="E15" t="inlineStr">
+      <c r="H15" t="inlineStr">
         <is>
           <t>crassipes</t>
         </is>
       </c>
-      <c r="F15" t="inlineStr">
+      <c r="J15" t="inlineStr">
         <is>
           <t>Hemsl.</t>
         </is>
       </c>
-      <c r="I15" t="inlineStr">
+      <c r="P15" t="b">
+        <v>1</v>
+      </c>
+      <c r="S15" t="inlineStr">
         <is>
           <t>Marsdenia crassipes</t>
         </is>
       </c>
-      <c r="J15" t="inlineStr">
+      <c r="T15" t="inlineStr">
         <is>
           <t>Marsdenia crassipes</t>
         </is>
       </c>
-      <c r="K15" t="inlineStr">
+      <c r="U15" t="inlineStr">
         <is>
           <t>Hemsl.</t>
         </is>
       </c>
-      <c r="L15" t="inlineStr">
-        <is>
-          <t>Species</t>
-        </is>
-      </c>
-      <c r="M15" t="inlineStr">
+      <c r="V15" t="inlineStr">
+        <is>
+          <t>Species</t>
+        </is>
+      </c>
+      <c r="W15" t="inlineStr">
         <is>
           <t>Synonym</t>
         </is>
       </c>
-      <c r="N15">
+      <c r="X15">
         <v>508007</v>
       </c>
-      <c r="O15" t="inlineStr">
+      <c r="Y15" t="inlineStr">
         <is>
           <t>99121-1</t>
         </is>
       </c>
-      <c r="P15">
-        <v>1</v>
-      </c>
-      <c r="Q15">
+      <c r="Z15">
+        <v>1</v>
+      </c>
+      <c r="AA15">
         <v>3308424</v>
       </c>
-      <c r="R15" t="inlineStr">
+      <c r="AB15" t="inlineStr">
         <is>
           <t>77311821-1</t>
         </is>
       </c>
-      <c r="S15" t="inlineStr">
+      <c r="AC15" t="inlineStr">
         <is>
           <t>77311821-1</t>
         </is>
       </c>
-      <c r="T15" t="inlineStr">
+      <c r="AD15" t="inlineStr">
         <is>
           <t>Ruehssia crassipes</t>
         </is>
       </c>
-      <c r="U15" t="inlineStr">
+      <c r="AE15" t="inlineStr">
         <is>
           <t>Ruehssia</t>
         </is>
       </c>
-      <c r="V15" t="inlineStr">
+      <c r="AF15" t="inlineStr">
         <is>
           <t>crassipes</t>
         </is>
       </c>
-      <c r="W15" t="inlineStr">
-        <is>
-          <t>Species</t>
-        </is>
-      </c>
-      <c r="X15" t="inlineStr">
+      <c r="AG15" t="inlineStr">
+        <is>
+          <t>Species</t>
+        </is>
+      </c>
+      <c r="AH15" t="inlineStr">
         <is>
           <t>Apocynaceae</t>
         </is>
       </c>
-      <c r="AA15" t="inlineStr">
+      <c r="AK15" t="inlineStr">
         <is>
           <t>Morillo &amp; Mora Méndez</t>
         </is>
       </c>
-      <c r="AB15" t="inlineStr">
+      <c r="AL15" t="inlineStr">
         <is>
           <t>(Hemsl.) Morillo &amp; Mora Méndez</t>
         </is>
       </c>
-      <c r="AC15" t="inlineStr">
+      <c r="AM15" t="inlineStr">
         <is>
           <t>climbing perennial</t>
         </is>
       </c>
-      <c r="AD15" t="b">
+      <c r="AN15" t="b">
         <v>1</v>
       </c>
     </row>
@@ -2153,106 +2275,106 @@
           <t>Metalepis peraffinis</t>
         </is>
       </c>
-      <c r="D16" t="inlineStr">
+      <c r="G16" t="inlineStr">
         <is>
           <t>Metalepis</t>
         </is>
       </c>
-      <c r="E16" t="inlineStr">
+      <c r="H16" t="inlineStr">
         <is>
           <t>peraffinis</t>
         </is>
       </c>
-      <c r="I16" t="inlineStr">
+      <c r="S16" t="inlineStr">
         <is>
           <t>Metalepis peraffinis</t>
         </is>
       </c>
-      <c r="J16" t="inlineStr">
+      <c r="T16" t="inlineStr">
         <is>
           <t>Metalepis peraffinis</t>
         </is>
       </c>
-      <c r="K16" t="inlineStr">
+      <c r="U16" t="inlineStr">
         <is>
           <t>(Woodson) Morillo</t>
         </is>
       </c>
-      <c r="L16" t="inlineStr">
-        <is>
-          <t>Species</t>
-        </is>
-      </c>
-      <c r="M16" t="inlineStr">
+      <c r="V16" t="inlineStr">
+        <is>
+          <t>Species</t>
+        </is>
+      </c>
+      <c r="W16" t="inlineStr">
         <is>
           <t>Synonym</t>
         </is>
       </c>
-      <c r="N16">
+      <c r="X16">
         <v>508813</v>
       </c>
-      <c r="O16" t="inlineStr">
+      <c r="Y16" t="inlineStr">
         <is>
           <t>963205-1</t>
         </is>
       </c>
-      <c r="P16">
-        <v>1</v>
-      </c>
-      <c r="Q16">
+      <c r="Z16">
+        <v>1</v>
+      </c>
+      <c r="AA16">
         <v>504030</v>
       </c>
-      <c r="R16" t="inlineStr">
+      <c r="AB16" t="inlineStr">
         <is>
           <t>310022-2</t>
         </is>
       </c>
-      <c r="S16" t="inlineStr">
+      <c r="AC16" t="inlineStr">
         <is>
           <t>310022-2</t>
         </is>
       </c>
-      <c r="T16" t="inlineStr">
+      <c r="AD16" t="inlineStr">
         <is>
           <t>Cynanchum peraffine</t>
         </is>
       </c>
-      <c r="U16" t="inlineStr">
+      <c r="AE16" t="inlineStr">
         <is>
           <t>Cynanchum</t>
         </is>
       </c>
-      <c r="V16" t="inlineStr">
+      <c r="AF16" t="inlineStr">
         <is>
           <t>peraffine</t>
         </is>
       </c>
-      <c r="W16" t="inlineStr">
-        <is>
-          <t>Species</t>
-        </is>
-      </c>
-      <c r="X16" t="inlineStr">
+      <c r="AG16" t="inlineStr">
+        <is>
+          <t>Species</t>
+        </is>
+      </c>
+      <c r="AH16" t="inlineStr">
         <is>
           <t>Apocynaceae</t>
         </is>
       </c>
-      <c r="AA16" t="inlineStr">
+      <c r="AK16" t="inlineStr">
         <is>
           <t>Woodson</t>
         </is>
       </c>
-      <c r="AB16" t="inlineStr">
+      <c r="AL16" t="inlineStr">
         <is>
           <t>Woodson</t>
         </is>
       </c>
-      <c r="AC16" t="inlineStr">
+      <c r="AM16" t="inlineStr">
         <is>
           <t>climbing subshrub</t>
         </is>
       </c>
-      <c r="AD16" t="b">
+      <c r="AN16" t="b">
         <v>1</v>
       </c>
     </row>
@@ -2269,114 +2391,147 @@
       </c>
       <c r="C17" t="inlineStr">
         <is>
+          <t>Pseudosicydium acariianthum</t>
+        </is>
+      </c>
+      <c r="D17" t="inlineStr">
+        <is>
+          <t>Pteropepon acariianthum</t>
+        </is>
+      </c>
+      <c r="E17" t="inlineStr">
+        <is>
+          <t>Pseudosicydium acariianthum</t>
+        </is>
+      </c>
+      <c r="F17" t="inlineStr">
+        <is>
           <t>Cucurbitaceae</t>
         </is>
       </c>
-      <c r="D17" t="inlineStr">
+      <c r="G17" t="inlineStr">
         <is>
           <t>Pteropepon</t>
         </is>
       </c>
-      <c r="E17" t="inlineStr">
+      <c r="H17" t="inlineStr">
         <is>
           <t>acariianthum</t>
         </is>
       </c>
-      <c r="F17" t="inlineStr">
+      <c r="J17" t="inlineStr">
         <is>
           <t>(Harms) H.Schaef. &amp; S.S. Renner</t>
         </is>
       </c>
-      <c r="I17" t="inlineStr">
+      <c r="L17" t="inlineStr">
+        <is>
+          <t>Pseudosicydium</t>
+        </is>
+      </c>
+      <c r="M17" t="inlineStr">
+        <is>
+          <t>acariianthum</t>
+        </is>
+      </c>
+      <c r="O17" t="inlineStr">
+        <is>
+          <t>Harms</t>
+        </is>
+      </c>
+      <c r="P17" t="b">
+        <v>1</v>
+      </c>
+      <c r="S17" t="inlineStr">
         <is>
           <t>Pteropepon acariianthum</t>
         </is>
       </c>
-      <c r="J17" t="inlineStr">
+      <c r="T17" t="inlineStr">
         <is>
           <t>Pteropepon acariaeanthus</t>
         </is>
       </c>
-      <c r="K17" t="inlineStr">
+      <c r="U17" t="inlineStr">
         <is>
           <t>(Harms) H.Schaef. &amp; S.S.Renner</t>
         </is>
       </c>
-      <c r="L17" t="inlineStr">
-        <is>
-          <t>Species</t>
-        </is>
-      </c>
-      <c r="M17" t="inlineStr">
+      <c r="V17" t="inlineStr">
+        <is>
+          <t>Species</t>
+        </is>
+      </c>
+      <c r="W17" t="inlineStr">
         <is>
           <t>Accepted</t>
         </is>
       </c>
-      <c r="N17">
+      <c r="X17">
         <v>2903160</v>
       </c>
-      <c r="O17" t="inlineStr">
+      <c r="Y17" t="inlineStr">
         <is>
           <t>77110583-1</t>
         </is>
       </c>
-      <c r="P17">
+      <c r="Z17">
         <v>0.875</v>
       </c>
-      <c r="Q17">
+      <c r="AA17">
         <v>2903160</v>
       </c>
-      <c r="R17" t="inlineStr">
+      <c r="AB17" t="inlineStr">
         <is>
           <t>77110583-1</t>
         </is>
       </c>
-      <c r="S17" t="inlineStr">
+      <c r="AC17" t="inlineStr">
         <is>
           <t>77110583-1</t>
         </is>
       </c>
-      <c r="T17" t="inlineStr">
+      <c r="AD17" t="inlineStr">
         <is>
           <t>Pteropepon acariaeanthus</t>
         </is>
       </c>
-      <c r="U17" t="inlineStr">
+      <c r="AE17" t="inlineStr">
         <is>
           <t>Pteropepon</t>
         </is>
       </c>
-      <c r="V17" t="inlineStr">
+      <c r="AF17" t="inlineStr">
         <is>
           <t>acariaeanthus</t>
         </is>
       </c>
-      <c r="W17" t="inlineStr">
-        <is>
-          <t>Species</t>
-        </is>
-      </c>
-      <c r="X17" t="inlineStr">
+      <c r="AG17" t="inlineStr">
+        <is>
+          <t>Species</t>
+        </is>
+      </c>
+      <c r="AH17" t="inlineStr">
         <is>
           <t>Cucurbitaceae</t>
         </is>
       </c>
-      <c r="AA17" t="inlineStr">
+      <c r="AK17" t="inlineStr">
         <is>
           <t>H.Schaef. &amp; S.S.Renner</t>
         </is>
       </c>
-      <c r="AB17" t="inlineStr">
+      <c r="AL17" t="inlineStr">
         <is>
           <t>(Harms) H.Schaef. &amp; S.S.Renner</t>
         </is>
       </c>
-      <c r="AC17" t="inlineStr">
+      <c r="AM17" t="inlineStr">
         <is>
           <t>liana</t>
         </is>
       </c>
-      <c r="AD17" t="b">
+      <c r="AN17" t="b">
         <v>0</v>
       </c>
     </row>
@@ -2393,114 +2548,147 @@
       </c>
       <c r="C18" t="inlineStr">
         <is>
+          <t>Acacia acanthopylla</t>
+        </is>
+      </c>
+      <c r="D18" t="inlineStr">
+        <is>
+          <t>Senegalia acanthopylla</t>
+        </is>
+      </c>
+      <c r="E18" t="inlineStr">
+        <is>
+          <t>Acacia acanthopylla</t>
+        </is>
+      </c>
+      <c r="F18" t="inlineStr">
+        <is>
           <t>Fabaceae</t>
         </is>
       </c>
-      <c r="D18" t="inlineStr">
+      <c r="G18" t="inlineStr">
         <is>
           <t>Senegalia</t>
         </is>
       </c>
-      <c r="E18" t="inlineStr">
+      <c r="H18" t="inlineStr">
         <is>
           <t>acanthopylla</t>
         </is>
       </c>
-      <c r="F18" t="inlineStr">
+      <c r="J18" t="inlineStr">
         <is>
           <t>Benth.(Britton &amp; Rose) Standl.».)</t>
         </is>
       </c>
-      <c r="I18" t="inlineStr">
+      <c r="L18" t="inlineStr">
+        <is>
+          <t>Acacia</t>
+        </is>
+      </c>
+      <c r="M18" t="inlineStr">
+        <is>
+          <t>acanthopylla</t>
+        </is>
+      </c>
+      <c r="O18" t="inlineStr">
+        <is>
+          <t>Britton &amp; Rose) Standl.</t>
+        </is>
+      </c>
+      <c r="P18" t="b">
+        <v>1</v>
+      </c>
+      <c r="S18" t="inlineStr">
         <is>
           <t>Senegalia acanthopylla</t>
         </is>
       </c>
-      <c r="J18" t="inlineStr">
+      <c r="T18" t="inlineStr">
         <is>
           <t>Senegalia acanthophylla</t>
         </is>
       </c>
-      <c r="K18" t="inlineStr">
+      <c r="U18" t="inlineStr">
         <is>
           <t>Britton &amp; Rose</t>
         </is>
       </c>
-      <c r="L18" t="inlineStr">
-        <is>
-          <t>Species</t>
-        </is>
-      </c>
-      <c r="M18" t="inlineStr">
+      <c r="V18" t="inlineStr">
+        <is>
+          <t>Species</t>
+        </is>
+      </c>
+      <c r="W18" t="inlineStr">
         <is>
           <t>Synonym</t>
         </is>
       </c>
-      <c r="N18">
+      <c r="X18">
         <v>2590663</v>
       </c>
-      <c r="O18" t="inlineStr">
+      <c r="Y18" t="inlineStr">
         <is>
           <t>518232-1</t>
         </is>
       </c>
-      <c r="P18">
+      <c r="Z18">
         <v>0.957</v>
       </c>
-      <c r="Q18">
+      <c r="AA18">
         <v>2590669</v>
       </c>
-      <c r="R18" t="inlineStr">
+      <c r="AB18" t="inlineStr">
         <is>
           <t>518260-1</t>
         </is>
       </c>
-      <c r="S18" t="inlineStr">
+      <c r="AC18" t="inlineStr">
         <is>
           <t>518260-1</t>
         </is>
       </c>
-      <c r="T18" t="inlineStr">
+      <c r="AD18" t="inlineStr">
         <is>
           <t>Senegalia hayesii</t>
         </is>
       </c>
-      <c r="U18" t="inlineStr">
+      <c r="AE18" t="inlineStr">
         <is>
           <t>Senegalia</t>
         </is>
       </c>
-      <c r="V18" t="inlineStr">
+      <c r="AF18" t="inlineStr">
         <is>
           <t>hayesii</t>
         </is>
       </c>
-      <c r="W18" t="inlineStr">
-        <is>
-          <t>Species</t>
-        </is>
-      </c>
-      <c r="X18" t="inlineStr">
+      <c r="AG18" t="inlineStr">
+        <is>
+          <t>Species</t>
+        </is>
+      </c>
+      <c r="AH18" t="inlineStr">
         <is>
           <t>Fabaceae</t>
         </is>
       </c>
-      <c r="AA18" t="inlineStr">
+      <c r="AK18" t="inlineStr">
         <is>
           <t>Britton &amp; Rose</t>
         </is>
       </c>
-      <c r="AB18" t="inlineStr">
+      <c r="AL18" t="inlineStr">
         <is>
           <t>(Benth.) Britton &amp; Rose</t>
         </is>
       </c>
-      <c r="AC18" t="inlineStr">
+      <c r="AM18" t="inlineStr">
         <is>
           <t>scrambling shrub or tree</t>
         </is>
       </c>
-      <c r="AD18" t="b">
+      <c r="AN18" t="b">
         <v>0</v>
       </c>
     </row>
@@ -2517,114 +2705,132 @@
       </c>
       <c r="C19" t="inlineStr">
         <is>
+          <t>NA NA</t>
+        </is>
+      </c>
+      <c r="D19" t="inlineStr">
+        <is>
+          <t>Smilax lanceolata</t>
+        </is>
+      </c>
+      <c r="E19" t="inlineStr">
+        <is>
+          <t>NA NA</t>
+        </is>
+      </c>
+      <c r="F19" t="inlineStr">
+        <is>
           <t>Smilacaceae</t>
         </is>
       </c>
-      <c r="D19" t="inlineStr">
+      <c r="G19" t="inlineStr">
         <is>
           <t>Smilax</t>
         </is>
       </c>
-      <c r="E19" t="inlineStr">
+      <c r="H19" t="inlineStr">
         <is>
           <t>lanceolata</t>
         </is>
       </c>
-      <c r="F19" t="inlineStr">
+      <c r="J19" t="inlineStr">
         <is>
           <t>Walter</t>
         </is>
       </c>
-      <c r="I19" t="inlineStr">
+      <c r="P19" t="b">
+        <v>1</v>
+      </c>
+      <c r="S19" t="inlineStr">
         <is>
           <t>Smilax lanceolata</t>
         </is>
       </c>
-      <c r="J19" t="inlineStr">
+      <c r="T19" t="inlineStr">
         <is>
           <t>Smilax lanceolata</t>
         </is>
       </c>
-      <c r="K19" t="inlineStr">
+      <c r="U19" t="inlineStr">
         <is>
           <t>L.</t>
         </is>
       </c>
-      <c r="L19" t="inlineStr">
-        <is>
-          <t>Species</t>
-        </is>
-      </c>
-      <c r="M19" t="inlineStr">
+      <c r="V19" t="inlineStr">
+        <is>
+          <t>Species</t>
+        </is>
+      </c>
+      <c r="W19" t="inlineStr">
         <is>
           <t>Synonym</t>
         </is>
       </c>
-      <c r="N19">
+      <c r="X19">
         <v>289209</v>
       </c>
-      <c r="O19" t="inlineStr">
+      <c r="Y19" t="inlineStr">
         <is>
           <t>541556-1</t>
         </is>
       </c>
-      <c r="P19">
-        <v>1</v>
-      </c>
-      <c r="Q19">
+      <c r="Z19">
+        <v>1</v>
+      </c>
+      <c r="AA19">
         <v>289271</v>
       </c>
-      <c r="R19" t="inlineStr">
+      <c r="AB19" t="inlineStr">
         <is>
           <t>317919-2</t>
         </is>
       </c>
-      <c r="S19" t="inlineStr">
+      <c r="AC19" t="inlineStr">
         <is>
           <t>317919-2</t>
         </is>
       </c>
-      <c r="T19" t="inlineStr">
+      <c r="AD19" t="inlineStr">
         <is>
           <t>Smilax laurifolia</t>
         </is>
       </c>
-      <c r="U19" t="inlineStr">
+      <c r="AE19" t="inlineStr">
         <is>
           <t>Smilax</t>
         </is>
       </c>
-      <c r="V19" t="inlineStr">
+      <c r="AF19" t="inlineStr">
         <is>
           <t>laurifolia</t>
         </is>
       </c>
-      <c r="W19" t="inlineStr">
-        <is>
-          <t>Species</t>
-        </is>
-      </c>
-      <c r="X19" t="inlineStr">
+      <c r="AG19" t="inlineStr">
+        <is>
+          <t>Species</t>
+        </is>
+      </c>
+      <c r="AH19" t="inlineStr">
         <is>
           <t>Smilacaceae</t>
         </is>
       </c>
-      <c r="AA19" t="inlineStr">
+      <c r="AK19" t="inlineStr">
         <is>
           <t>L.</t>
         </is>
       </c>
-      <c r="AB19" t="inlineStr">
+      <c r="AL19" t="inlineStr">
         <is>
           <t>L.</t>
         </is>
       </c>
-      <c r="AC19" t="inlineStr">
+      <c r="AM19" t="inlineStr">
         <is>
           <t>tuberous hydrogeophyte</t>
         </is>
       </c>
-      <c r="AD19" t="b">
+      <c r="AN19" t="b">
         <v>1</v>
       </c>
     </row>
@@ -2641,114 +2847,132 @@
       </c>
       <c r="C20" t="inlineStr">
         <is>
+          <t>NA NA</t>
+        </is>
+      </c>
+      <c r="D20" t="inlineStr">
+        <is>
+          <t>Smilax panamensis</t>
+        </is>
+      </c>
+      <c r="E20" t="inlineStr">
+        <is>
+          <t>NA NA</t>
+        </is>
+      </c>
+      <c r="F20" t="inlineStr">
+        <is>
           <t>Smilacaceae</t>
         </is>
       </c>
-      <c r="D20" t="inlineStr">
+      <c r="G20" t="inlineStr">
         <is>
           <t>Smilax</t>
         </is>
       </c>
-      <c r="E20" t="inlineStr">
+      <c r="H20" t="inlineStr">
         <is>
           <t>panamensis</t>
         </is>
       </c>
-      <c r="F20" t="inlineStr">
+      <c r="J20" t="inlineStr">
         <is>
           <t>Morong</t>
         </is>
       </c>
-      <c r="I20" t="inlineStr">
+      <c r="P20" t="b">
+        <v>1</v>
+      </c>
+      <c r="S20" t="inlineStr">
         <is>
           <t>Smilax panamensis</t>
         </is>
       </c>
-      <c r="J20" t="inlineStr">
+      <c r="T20" t="inlineStr">
         <is>
           <t>Smilax panamensis</t>
         </is>
       </c>
-      <c r="K20" t="inlineStr">
+      <c r="U20" t="inlineStr">
         <is>
           <t>Morong</t>
         </is>
       </c>
-      <c r="L20" t="inlineStr">
-        <is>
-          <t>Species</t>
-        </is>
-      </c>
-      <c r="M20" t="inlineStr">
+      <c r="V20" t="inlineStr">
+        <is>
+          <t>Species</t>
+        </is>
+      </c>
+      <c r="W20" t="inlineStr">
         <is>
           <t>Synonym</t>
         </is>
       </c>
-      <c r="N20">
+      <c r="X20">
         <v>288944</v>
       </c>
-      <c r="O20" t="inlineStr">
+      <c r="Y20" t="inlineStr">
         <is>
           <t>237989-2</t>
         </is>
       </c>
-      <c r="P20">
-        <v>1</v>
-      </c>
-      <c r="Q20">
+      <c r="Z20">
+        <v>1</v>
+      </c>
+      <c r="AA20">
         <v>288875</v>
       </c>
-      <c r="R20" t="inlineStr">
+      <c r="AB20" t="inlineStr">
         <is>
           <t>541778-1</t>
         </is>
       </c>
-      <c r="S20" t="inlineStr">
+      <c r="AC20" t="inlineStr">
         <is>
           <t>541778-1</t>
         </is>
       </c>
-      <c r="T20" t="inlineStr">
+      <c r="AD20" t="inlineStr">
         <is>
           <t>Smilax purhampuy</t>
         </is>
       </c>
-      <c r="U20" t="inlineStr">
+      <c r="AE20" t="inlineStr">
         <is>
           <t>Smilax</t>
         </is>
       </c>
-      <c r="V20" t="inlineStr">
+      <c r="AF20" t="inlineStr">
         <is>
           <t>purhampuy</t>
         </is>
       </c>
-      <c r="W20" t="inlineStr">
-        <is>
-          <t>Species</t>
-        </is>
-      </c>
-      <c r="X20" t="inlineStr">
+      <c r="AG20" t="inlineStr">
+        <is>
+          <t>Species</t>
+        </is>
+      </c>
+      <c r="AH20" t="inlineStr">
         <is>
           <t>Smilacaceae</t>
         </is>
       </c>
-      <c r="AA20" t="inlineStr">
+      <c r="AK20" t="inlineStr">
         <is>
           <t>Ruiz</t>
         </is>
       </c>
-      <c r="AB20" t="inlineStr">
+      <c r="AL20" t="inlineStr">
         <is>
           <t>Ruiz</t>
         </is>
       </c>
-      <c r="AC20" t="inlineStr">
+      <c r="AM20" t="inlineStr">
         <is>
           <t>climber</t>
         </is>
       </c>
-      <c r="AD20" t="b">
+      <c r="AN20" t="b">
         <v>1</v>
       </c>
     </row>
@@ -2763,106 +2987,106 @@
           <t>Tontelea richardii</t>
         </is>
       </c>
-      <c r="D21" t="inlineStr">
+      <c r="G21" t="inlineStr">
         <is>
           <t>Tontelea</t>
         </is>
       </c>
-      <c r="E21" t="inlineStr">
+      <c r="H21" t="inlineStr">
         <is>
           <t>richardii</t>
         </is>
       </c>
-      <c r="I21" t="inlineStr">
+      <c r="S21" t="inlineStr">
         <is>
           <t>Tontelea richardii</t>
         </is>
       </c>
-      <c r="J21" t="inlineStr">
+      <c r="T21" t="inlineStr">
         <is>
           <t>Tontelea richardii</t>
         </is>
       </c>
-      <c r="K21" t="inlineStr">
+      <c r="U21" t="inlineStr">
         <is>
           <t>(Peyr.) A.C.Sm.</t>
         </is>
       </c>
-      <c r="L21" t="inlineStr">
-        <is>
-          <t>Species</t>
-        </is>
-      </c>
-      <c r="M21" t="inlineStr">
+      <c r="V21" t="inlineStr">
+        <is>
+          <t>Species</t>
+        </is>
+      </c>
+      <c r="W21" t="inlineStr">
         <is>
           <t>Synonym</t>
         </is>
       </c>
-      <c r="N21">
+      <c r="X21">
         <v>2443071</v>
       </c>
-      <c r="O21" t="inlineStr">
+      <c r="Y21" t="inlineStr">
         <is>
           <t>255084-2</t>
         </is>
       </c>
-      <c r="P21">
-        <v>1</v>
-      </c>
-      <c r="Q21">
+      <c r="Z21">
+        <v>1</v>
+      </c>
+      <c r="AA21">
         <v>2905292</v>
       </c>
-      <c r="R21" t="inlineStr">
+      <c r="AB21" t="inlineStr">
         <is>
           <t>77112015-1</t>
         </is>
       </c>
-      <c r="S21" t="inlineStr">
+      <c r="AC21" t="inlineStr">
         <is>
           <t>77112015-1</t>
         </is>
       </c>
-      <c r="T21" t="inlineStr">
+      <c r="AD21" t="inlineStr">
         <is>
           <t>Tontelea passiflora</t>
         </is>
       </c>
-      <c r="U21" t="inlineStr">
+      <c r="AE21" t="inlineStr">
         <is>
           <t>Tontelea</t>
         </is>
       </c>
-      <c r="V21" t="inlineStr">
+      <c r="AF21" t="inlineStr">
         <is>
           <t>passiflora</t>
         </is>
       </c>
-      <c r="W21" t="inlineStr">
-        <is>
-          <t>Species</t>
-        </is>
-      </c>
-      <c r="X21" t="inlineStr">
+      <c r="AG21" t="inlineStr">
+        <is>
+          <t>Species</t>
+        </is>
+      </c>
+      <c r="AH21" t="inlineStr">
         <is>
           <t>Celastraceae</t>
         </is>
       </c>
-      <c r="AA21" t="inlineStr">
+      <c r="AK21" t="inlineStr">
         <is>
           <t>Lombardi</t>
         </is>
       </c>
-      <c r="AB21" t="inlineStr">
+      <c r="AL21" t="inlineStr">
         <is>
           <t>(Vell.) Lombardi</t>
         </is>
       </c>
-      <c r="AC21" t="inlineStr">
+      <c r="AM21" t="inlineStr">
         <is>
           <t>scrambling shrub or tree</t>
         </is>
       </c>
-      <c r="AD21" t="b">
+      <c r="AN21" t="b">
         <v>1</v>
       </c>
     </row>
@@ -2879,114 +3103,132 @@
       </c>
       <c r="C22" t="inlineStr">
         <is>
+          <t>NA NA</t>
+        </is>
+      </c>
+      <c r="D22" t="inlineStr">
+        <is>
+          <t>Urera eggersii</t>
+        </is>
+      </c>
+      <c r="E22" t="inlineStr">
+        <is>
+          <t>NA NA</t>
+        </is>
+      </c>
+      <c r="F22" t="inlineStr">
+        <is>
           <t>Urticaceae</t>
         </is>
       </c>
-      <c r="D22" t="inlineStr">
+      <c r="G22" t="inlineStr">
         <is>
           <t>Urera</t>
         </is>
       </c>
-      <c r="E22" t="inlineStr">
+      <c r="H22" t="inlineStr">
         <is>
           <t>eggersii</t>
         </is>
       </c>
-      <c r="F22" t="inlineStr">
+      <c r="J22" t="inlineStr">
         <is>
           <t>Hieron.</t>
         </is>
       </c>
-      <c r="I22" t="inlineStr">
+      <c r="P22" t="b">
+        <v>1</v>
+      </c>
+      <c r="S22" t="inlineStr">
         <is>
           <t>Urera eggersii</t>
         </is>
       </c>
-      <c r="J22" t="inlineStr">
+      <c r="T22" t="inlineStr">
         <is>
           <t>Urera eggersii</t>
         </is>
       </c>
-      <c r="K22" t="inlineStr">
+      <c r="U22" t="inlineStr">
         <is>
           <t>Hieron.</t>
         </is>
       </c>
-      <c r="L22" t="inlineStr">
-        <is>
-          <t>Species</t>
-        </is>
-      </c>
-      <c r="M22" t="inlineStr">
+      <c r="V22" t="inlineStr">
+        <is>
+          <t>Species</t>
+        </is>
+      </c>
+      <c r="W22" t="inlineStr">
         <is>
           <t>Synonym</t>
         </is>
       </c>
-      <c r="N22">
+      <c r="X22">
         <v>2448453</v>
       </c>
-      <c r="O22" t="inlineStr">
+      <c r="Y22" t="inlineStr">
         <is>
           <t>261643-2</t>
         </is>
       </c>
-      <c r="P22">
-        <v>1</v>
-      </c>
-      <c r="Q22">
+      <c r="Z22">
+        <v>1</v>
+      </c>
+      <c r="AA22">
         <v>2446483</v>
       </c>
-      <c r="R22" t="inlineStr">
+      <c r="AB22" t="inlineStr">
         <is>
           <t>857063-1</t>
         </is>
       </c>
-      <c r="S22" t="inlineStr">
+      <c r="AC22" t="inlineStr">
         <is>
           <t>857063-1</t>
         </is>
       </c>
-      <c r="T22" t="inlineStr">
+      <c r="AD22" t="inlineStr">
         <is>
           <t>Urera simplex</t>
         </is>
       </c>
-      <c r="U22" t="inlineStr">
+      <c r="AE22" t="inlineStr">
         <is>
           <t>Urera</t>
         </is>
       </c>
-      <c r="V22" t="inlineStr">
+      <c r="AF22" t="inlineStr">
         <is>
           <t>simplex</t>
         </is>
       </c>
-      <c r="W22" t="inlineStr">
-        <is>
-          <t>Species</t>
-        </is>
-      </c>
-      <c r="X22" t="inlineStr">
+      <c r="AG22" t="inlineStr">
+        <is>
+          <t>Species</t>
+        </is>
+      </c>
+      <c r="AH22" t="inlineStr">
         <is>
           <t>Urticaceae</t>
         </is>
       </c>
-      <c r="AA22" t="inlineStr">
+      <c r="AK22" t="inlineStr">
         <is>
           <t>Wedd.</t>
         </is>
       </c>
-      <c r="AB22" t="inlineStr">
+      <c r="AL22" t="inlineStr">
         <is>
           <t>Wedd.</t>
         </is>
       </c>
-      <c r="AC22" t="inlineStr">
+      <c r="AM22" t="inlineStr">
         <is>
           <t>scrambling shrub or tree</t>
         </is>
       </c>
-      <c r="AD22" t="b">
+      <c r="AN22" t="b">
         <v>1</v>
       </c>
     </row>

</xml_diff>